<commit_message>
Update 90-day plan xlsx
Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SMBX_90_DAY_PLAN.xlsx
+++ b/SMBX_90_DAY_PLAN.xlsx
@@ -614,7 +614,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -674,7 +674,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>DEALFLOW NETWORK (152K)</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>SuperCFO Group (262K)</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -794,7 +794,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Small Business Network (314K)</t>
+          <t>Business Owners &amp; Investors Network (1.8M)</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -1814,7 +1814,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Investment Bankers Group (40K)</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Private Equity &amp; Hedge Fund (152K)</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1934,7 +1934,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Family Offices &amp; Institutional Investors (60K)</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1994,7 +1994,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>The Founders Exchange (259K)</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -3014,7 +3014,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>DEALFLOW NETWORK (152K)</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -3074,7 +3074,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Institutional Investors &amp; Allocators (88K)</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -3134,7 +3134,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Investment Banking BA &amp; PM (188K)</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Chief Executive Officer &amp; Leadership (54K)</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -4274,7 +4274,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Deal Maker Club (49K)</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -4334,7 +4334,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Finance &amp; Banking Fintech (1M)</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Leadership Think Tank (2.2M)</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Deal Maker Club (49K)</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -5474,7 +5474,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -5534,7 +5534,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>SuperCFO Group (262K)</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Business Owners &amp; Investors Network (1.8M)</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -6614,7 +6614,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Private Equity &amp; Hedge Fund (152K)</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Investment Bankers Group (40K)</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -6734,7 +6734,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Banking &amp; Finance (285K)</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -6794,7 +6794,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>The Founders Exchange (259K)</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -7814,7 +7814,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Institutional Investors &amp; Allocators (88K)</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -7874,7 +7874,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>DEALFLOW NETWORK (152K)</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -7934,7 +7934,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Family Offices &amp; Institutional Investors (60K)</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -7994,7 +7994,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Chief Executive Officer &amp; Leadership (54K)</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -9014,7 +9014,7 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>M&amp;A and Corporate Finance Europe (24K)</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -9074,7 +9074,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Private Equity &amp; Hedge Fund (152K)</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -9134,7 +9134,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Investment Banking BA &amp; PM (188K)</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
@@ -9194,7 +9194,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Leadership Think Tank (2.2M)</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
@@ -10214,7 +10214,7 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -10274,7 +10274,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>DEALFLOW NETWORK (152K)</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -10334,7 +10334,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>SuperCFO Group (262K)</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -10394,7 +10394,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Business Owners &amp; Investors Network (1.8M)</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -11414,7 +11414,7 @@
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Investment Bankers Group (40K)</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -11474,7 +11474,7 @@
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Institutional Investors &amp; Allocators (88K)</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
@@ -11534,7 +11534,7 @@
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Finance &amp; Banking Fintech (1M)</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -11594,7 +11594,7 @@
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>The Founders Exchange (259K)</t>
         </is>
       </c>
       <c r="F185" s="2" t="inlineStr">
@@ -12614,7 +12614,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>DEALFLOW NETWORK (152K)</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
@@ -12674,7 +12674,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Deal Maker Club (49K)</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
@@ -12734,7 +12734,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Family Offices &amp; Institutional Investors (60K)</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
@@ -12794,7 +12794,7 @@
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Chief Executive Officer &amp; Leadership (54K)</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
@@ -13814,7 +13814,7 @@
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
@@ -13874,7 +13874,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Private Equity &amp; Hedge Fund (152K)</t>
         </is>
       </c>
       <c r="F223" s="2" t="inlineStr">
@@ -13934,7 +13934,7 @@
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Banking &amp; Finance (285K)</t>
         </is>
       </c>
       <c r="F224" s="2" t="inlineStr">
@@ -13994,7 +13994,7 @@
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Leadership Think Tank (2.2M)</t>
         </is>
       </c>
       <c r="F225" s="2" t="inlineStr">
@@ -15014,7 +15014,7 @@
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>SearchFunder (9.4K)</t>
+          <t>Deal Maker Club (49K)</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
@@ -15074,7 +15074,7 @@
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>PE/M&amp;A/VC (240K)</t>
+          <t>Mergers &amp; Acquisitions Network (283K)</t>
         </is>
       </c>
       <c r="F243" s="2" t="inlineStr">
@@ -15134,7 +15134,7 @@
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>VC Funds (46.5K)</t>
+          <t>Investment Banking BA &amp; PM (188K)</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
@@ -15194,7 +15194,7 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>Executive Suite (380K)</t>
+          <t>Business Owners &amp; Investors Network (1.8M)</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">

</xml_diff>